<commit_message>
inventory successfully imported to excel
</commit_message>
<xml_diff>
--- a/inStockInventory.xlsx
+++ b/inStockInventory.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,6 +529,59 @@
           <t>AS30188</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BEIGE</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AS30188</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BLACK</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AS30188</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>BROWN</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AS30188</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TAUPE</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="19">
       <c r="E19" t="inlineStr">
@@ -536,12 +589,133 @@
           <t>AS60158 SET</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>BG</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>AS60158 SET</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>AS60158 SET</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>AS60158 SET</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>KHA</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="36">
       <c r="E36" t="inlineStr">
         <is>
           <t>CR20202</t>
         </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>BK</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>GY</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>RBL</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>RUST</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>CR20202</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed excel and fixed images
</commit_message>
<xml_diff>
--- a/inStockInventory.xlsx
+++ b/inStockInventory.xlsx
@@ -155,7 +155,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3095625" cy="4371975"/>
@@ -180,7 +180,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>35</row>
+      <row>51</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3095625" cy="4381500"/>
@@ -493,13 +493,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
@@ -593,138 +593,138 @@
         <v>101</v>
       </c>
     </row>
-    <row r="19">
-      <c r="E19" t="inlineStr">
+    <row r="27">
+      <c r="E27" t="inlineStr">
         <is>
           <t>AS60158 SET</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>BG</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G27" t="n">
         <v>117</v>
       </c>
     </row>
-    <row r="20">
-      <c r="E20" t="inlineStr">
+    <row r="28">
+      <c r="E28" t="inlineStr">
         <is>
           <t>AS60158 SET</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>BK</t>
         </is>
       </c>
-      <c r="G20" t="n">
+      <c r="G28" t="n">
         <v>357</v>
       </c>
     </row>
-    <row r="21">
-      <c r="E21" t="inlineStr">
+    <row r="29">
+      <c r="E29" t="inlineStr">
         <is>
           <t>AS60158 SET</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="G21" t="n">
+      <c r="G29" t="n">
         <v>174</v>
       </c>
     </row>
-    <row r="22">
-      <c r="E22" t="inlineStr">
+    <row r="30">
+      <c r="E30" t="inlineStr">
         <is>
           <t>AS60158 SET</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>KHA</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="G30" t="n">
         <v>113</v>
       </c>
     </row>
-    <row r="36">
-      <c r="E36" t="inlineStr">
+    <row r="52">
+      <c r="E52" t="inlineStr">
         <is>
           <t>CR20202</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>BK</t>
         </is>
       </c>
-      <c r="G36" t="n">
+      <c r="G52" t="n">
         <v>163</v>
       </c>
     </row>
-    <row r="37">
-      <c r="E37" t="inlineStr">
+    <row r="53">
+      <c r="E53" t="inlineStr">
         <is>
           <t>CR20202</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>GY</t>
         </is>
       </c>
-      <c r="G37" t="n">
+      <c r="G53" t="n">
         <v>89</v>
       </c>
     </row>
-    <row r="38">
-      <c r="E38" t="inlineStr">
+    <row r="54">
+      <c r="E54" t="inlineStr">
         <is>
           <t>CR20202</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>RBL</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="G54" t="n">
         <v>98</v>
       </c>
     </row>
-    <row r="39">
-      <c r="E39" t="inlineStr">
+    <row r="55">
+      <c r="E55" t="inlineStr">
         <is>
           <t>CR20202</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>RUST</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="G55" t="n">
         <v>62</v>
       </c>
     </row>
-    <row r="40">
-      <c r="E40" t="inlineStr">
+    <row r="56">
+      <c r="E56" t="inlineStr">
         <is>
           <t>CR20202</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>TP</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G56" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>